<commit_message>
Stock en tres colores (rojo, amarillo, verde) con avisos por producto y por tipo
- Niveles automáticos por tipo de producto (bebidas, snacks, quesos por kilo, etc.), rotación y ventas
- El dueño los cambia por tipo (Ajustes) o por producto (Editar → Más opciones); columna StockAviso en Excel
- Pedido al proveedor: los rojos van solos y los amarillos se agregan con un toque
- Inicio, Productos y Vender muestran los tres colores; warn_stock en Supabase
- Arregla npm run ejemplo (import con .ts)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/ejemplo-inventario.xlsx
+++ b/public/ejemplo-inventario.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:J69"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="37.83203125" customWidth="1"/>
@@ -410,6 +410,7 @@
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
     <col min="8" max="8" width="8.83203125" customWidth="1"/>
     <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,6 +441,9 @@
       <c r="I1" t="str">
         <v>StockMinimo</v>
       </c>
+      <c r="J1" t="str">
+        <v>StockAviso</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -469,6 +473,9 @@
       <c r="I2" t="str">
         <v/>
       </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -498,6 +505,9 @@
       <c r="I3" t="str">
         <v/>
       </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -527,6 +537,9 @@
       <c r="I4" t="str">
         <v/>
       </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -556,6 +569,9 @@
       <c r="I5" t="str">
         <v/>
       </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -585,6 +601,9 @@
       <c r="I6" t="str">
         <v/>
       </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -614,6 +633,9 @@
       <c r="I7" t="str">
         <v/>
       </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -643,6 +665,9 @@
       <c r="I8" t="str">
         <v/>
       </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -672,6 +697,9 @@
       <c r="I9" t="str">
         <v/>
       </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -701,6 +729,9 @@
       <c r="I10" t="str">
         <v/>
       </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -730,6 +761,9 @@
       <c r="I11" t="str">
         <v/>
       </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -759,6 +793,9 @@
       <c r="I12" t="str">
         <v/>
       </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -788,6 +825,9 @@
       <c r="I13" t="str">
         <v/>
       </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -817,6 +857,9 @@
       <c r="I14" t="str">
         <v/>
       </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -846,6 +889,9 @@
       <c r="I15" t="str">
         <v/>
       </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -875,6 +921,9 @@
       <c r="I16" t="str">
         <v/>
       </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -904,6 +953,9 @@
       <c r="I17" t="str">
         <v/>
       </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -933,6 +985,9 @@
       <c r="I18" t="str">
         <v/>
       </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -962,6 +1017,9 @@
       <c r="I19" t="str">
         <v/>
       </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -991,6 +1049,9 @@
       <c r="I20" t="str">
         <v/>
       </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1020,6 +1081,9 @@
       <c r="I21" t="str">
         <v/>
       </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1049,6 +1113,9 @@
       <c r="I22" t="str">
         <v/>
       </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1078,6 +1145,9 @@
       <c r="I23" t="str">
         <v/>
       </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1107,6 +1177,9 @@
       <c r="I24" t="str">
         <v/>
       </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1136,6 +1209,9 @@
       <c r="I25" t="str">
         <v/>
       </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1165,6 +1241,9 @@
       <c r="I26" t="str">
         <v/>
       </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1194,6 +1273,9 @@
       <c r="I27" t="str">
         <v/>
       </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1223,6 +1305,9 @@
       <c r="I28" t="str">
         <v/>
       </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1252,6 +1337,9 @@
       <c r="I29" t="str">
         <v/>
       </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1281,6 +1369,9 @@
       <c r="I30" t="str">
         <v/>
       </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1310,6 +1401,9 @@
       <c r="I31" t="str">
         <v/>
       </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1339,6 +1433,9 @@
       <c r="I32" t="str">
         <v/>
       </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1368,6 +1465,9 @@
       <c r="I33" t="str">
         <v/>
       </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1397,6 +1497,9 @@
       <c r="I34" t="str">
         <v/>
       </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1426,6 +1529,9 @@
       <c r="I35" t="str">
         <v/>
       </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1455,6 +1561,9 @@
       <c r="I36" t="str">
         <v/>
       </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1484,6 +1593,9 @@
       <c r="I37" t="str">
         <v/>
       </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1513,6 +1625,9 @@
       <c r="I38" t="str">
         <v/>
       </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1542,6 +1657,9 @@
       <c r="I39" t="str">
         <v/>
       </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1571,6 +1689,9 @@
       <c r="I40" t="str">
         <v/>
       </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1600,6 +1721,9 @@
       <c r="I41" t="str">
         <v/>
       </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1629,6 +1753,9 @@
       <c r="I42" t="str">
         <v/>
       </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1658,6 +1785,9 @@
       <c r="I43" t="str">
         <v/>
       </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1687,6 +1817,9 @@
       <c r="I44" t="str">
         <v/>
       </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1716,6 +1849,9 @@
       <c r="I45" t="str">
         <v/>
       </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1745,6 +1881,9 @@
       <c r="I46" t="str">
         <v/>
       </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1774,6 +1913,9 @@
       <c r="I47" t="str">
         <v/>
       </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1803,6 +1945,9 @@
       <c r="I48" t="str">
         <v/>
       </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1832,6 +1977,9 @@
       <c r="I49" t="str">
         <v/>
       </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1861,6 +2009,9 @@
       <c r="I50" t="str">
         <v/>
       </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1890,6 +2041,9 @@
       <c r="I51" t="str">
         <v/>
       </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1919,6 +2073,9 @@
       <c r="I52" t="str">
         <v/>
       </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1948,6 +2105,9 @@
       <c r="I53" t="str">
         <v/>
       </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1977,6 +2137,9 @@
       <c r="I54" t="str">
         <v/>
       </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2006,6 +2169,9 @@
       <c r="I55" t="str">
         <v/>
       </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2035,6 +2201,9 @@
       <c r="I56" t="str">
         <v/>
       </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2064,6 +2233,9 @@
       <c r="I57" t="str">
         <v/>
       </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2093,6 +2265,9 @@
       <c r="I58" t="str">
         <v/>
       </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2122,6 +2297,9 @@
       <c r="I59" t="str">
         <v/>
       </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2151,6 +2329,9 @@
       <c r="I60" t="str">
         <v/>
       </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2180,6 +2361,9 @@
       <c r="I61" t="str">
         <v/>
       </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2209,6 +2393,9 @@
       <c r="I62" t="str">
         <v/>
       </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2238,6 +2425,9 @@
       <c r="I63" t="str">
         <v/>
       </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2267,6 +2457,9 @@
       <c r="I64" t="str">
         <v/>
       </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2296,6 +2489,9 @@
       <c r="I65" t="str">
         <v/>
       </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2325,6 +2521,9 @@
       <c r="I66" t="str">
         <v/>
       </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2354,6 +2553,9 @@
       <c r="I67" t="str">
         <v/>
       </c>
+      <c r="J67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2383,6 +2585,9 @@
       <c r="I68" t="str">
         <v/>
       </c>
+      <c r="J68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2412,10 +2617,13 @@
       <c r="I69" t="str">
         <v/>
       </c>
+      <c r="J69" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J69"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>